<commit_message>
୧ʕ•̀ᴥ•́ʔ୨ Edicion readme y pruebas AUTOMAP
</commit_message>
<xml_diff>
--- a/AUTOMAP/chip_layout_normalized.xlsx
+++ b/AUTOMAP/chip_layout_normalized.xlsx
@@ -8,22 +8,175 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\lab_repos\SurugaSeikiHex\AUTOMAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269DA9E2-010D-46F1-BB29-5A19723FA44B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19356D25-DA4D-41C2-AE54-FA45C0580533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
     <sheet name="Devices" sheetId="2" r:id="rId2"/>
     <sheet name="Ports" sheetId="3" r:id="rId3"/>
-    <sheet name="MeasurementPlan" sheetId="4" r:id="rId4"/>
+    <sheet name="Measurements" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="81">
+  <si>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>Port</t>
+  </si>
+  <si>
+    <t>Direction</t>
+  </si>
+  <si>
+    <t>X (um)</t>
+  </si>
+  <si>
+    <t>Y (um)</t>
+  </si>
+  <si>
+    <t>Coupling</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>MZI_01</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>Grating</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>OUT</t>
+  </si>
+  <si>
+    <t>Output</t>
+  </si>
+  <si>
+    <t>MMI_01</t>
+  </si>
+  <si>
+    <t>Edge</t>
+  </si>
+  <si>
+    <t>Output 1</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>Output 2</t>
+  </si>
+  <si>
+    <t>BTS_01</t>
+  </si>
+  <si>
+    <t>P4</t>
+  </si>
+  <si>
+    <t>Output 3</t>
+  </si>
+  <si>
+    <t>P5</t>
+  </si>
+  <si>
+    <t>Output 4</t>
+  </si>
+  <si>
+    <t>P6</t>
+  </si>
+  <si>
+    <t>Output 5</t>
+  </si>
+  <si>
+    <t>P7</t>
+  </si>
+  <si>
+    <t>Output 6</t>
+  </si>
+  <si>
+    <t>P8</t>
+  </si>
+  <si>
+    <t>Output 7</t>
+  </si>
+  <si>
+    <t>P9</t>
+  </si>
+  <si>
+    <t>Output 8</t>
+  </si>
+  <si>
+    <t>P10</t>
+  </si>
+  <si>
+    <t>Output 9</t>
+  </si>
+  <si>
+    <t>P11</t>
+  </si>
+  <si>
+    <t>Output 10</t>
+  </si>
+  <si>
+    <t>P12</t>
+  </si>
+  <si>
+    <t>Output 11</t>
+  </si>
+  <si>
+    <t>P13</t>
+  </si>
+  <si>
+    <t>Output 12</t>
+  </si>
+  <si>
+    <t>P14</t>
+  </si>
+  <si>
+    <t>Output 13</t>
+  </si>
+  <si>
+    <t>P15</t>
+  </si>
+  <si>
+    <t>Output 14</t>
+  </si>
+  <si>
+    <t>P16</t>
+  </si>
+  <si>
+    <t>Output 15</t>
+  </si>
+  <si>
+    <t>P17</t>
+  </si>
+  <si>
+    <t>Output 16</t>
+  </si>
+  <si>
+    <t>MMI_02</t>
+  </si>
+  <si>
+    <t>nan</t>
+  </si>
   <si>
     <t>Parameter</t>
   </si>
@@ -67,203 +220,59 @@
     <t>Example using normalized device/port model</t>
   </si>
   <si>
-    <t>Device</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
     <t>Description</t>
   </si>
   <si>
-    <t>MZI_01</t>
-  </si>
-  <si>
     <t>MZI</t>
   </si>
   <si>
     <t>Reference Mach-Zehnder</t>
   </si>
   <si>
-    <t>MMI_01</t>
-  </si>
-  <si>
     <t>MMI1x2</t>
   </si>
   <si>
     <t>1x2 splitter</t>
   </si>
   <si>
-    <t>BTS_01</t>
-  </si>
-  <si>
     <t>BTS1x16</t>
   </si>
   <si>
     <t>Binary Tree Splitter</t>
   </si>
   <si>
-    <t>Port</t>
-  </si>
-  <si>
-    <t>Direction</t>
-  </si>
-  <si>
-    <t>X (um)</t>
-  </si>
-  <si>
-    <t>Y (um)</t>
-  </si>
-  <si>
-    <t>Coupling</t>
-  </si>
-  <si>
-    <t>Comments</t>
-  </si>
-  <si>
-    <t>P1</t>
-  </si>
-  <si>
-    <t>IN</t>
-  </si>
-  <si>
-    <t>Grating</t>
-  </si>
-  <si>
-    <t>Input</t>
-  </si>
-  <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>OUT</t>
-  </si>
-  <si>
-    <t>Output</t>
-  </si>
-  <si>
-    <t>Edge</t>
-  </si>
-  <si>
-    <t>Output 1</t>
-  </si>
-  <si>
-    <t>P3</t>
-  </si>
-  <si>
-    <t>Output 2</t>
-  </si>
-  <si>
-    <t>P4</t>
-  </si>
-  <si>
-    <t>Output 3</t>
-  </si>
-  <si>
-    <t>P5</t>
-  </si>
-  <si>
-    <t>Output 4</t>
-  </si>
-  <si>
-    <t>P6</t>
-  </si>
-  <si>
-    <t>Output 5</t>
-  </si>
-  <si>
-    <t>P7</t>
-  </si>
-  <si>
-    <t>Output 6</t>
-  </si>
-  <si>
-    <t>P8</t>
-  </si>
-  <si>
-    <t>Output 7</t>
-  </si>
-  <si>
-    <t>P9</t>
-  </si>
-  <si>
-    <t>Output 8</t>
-  </si>
-  <si>
-    <t>P10</t>
-  </si>
-  <si>
-    <t>Output 9</t>
-  </si>
-  <si>
-    <t>P11</t>
-  </si>
-  <si>
-    <t>Output 10</t>
-  </si>
-  <si>
-    <t>P12</t>
-  </si>
-  <si>
-    <t>Output 11</t>
-  </si>
-  <si>
-    <t>P13</t>
-  </si>
-  <si>
-    <t>Output 12</t>
-  </si>
-  <si>
-    <t>P14</t>
-  </si>
-  <si>
-    <t>Output 13</t>
-  </si>
-  <si>
-    <t>P15</t>
-  </si>
-  <si>
-    <t>Output 14</t>
-  </si>
-  <si>
-    <t>P16</t>
-  </si>
-  <si>
-    <t>Output 15</t>
-  </si>
-  <si>
-    <t>P17</t>
-  </si>
-  <si>
-    <t>Output 16</t>
+    <t>MMI2X2</t>
+  </si>
+  <si>
+    <t>2x2 splitter</t>
   </si>
   <si>
     <t>Enabled</t>
   </si>
   <si>
-    <t>Priority</t>
+    <t>Status</t>
   </si>
   <si>
     <t>YES</t>
   </si>
   <si>
-    <t>MMI_02</t>
-  </si>
-  <si>
-    <t>MMI2X2</t>
-  </si>
-  <si>
-    <t>2x2 splitter</t>
-  </si>
-  <si>
-    <t>nan</t>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Measure</t>
+  </si>
+  <si>
+    <t>NO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -275,6 +284,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -297,14 +314,68 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -315,6 +386,58 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{504DE116-4C50-4705-9A3E-BE8293DC825F}" name="Table1" displayName="Table1" ref="A1:D5" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:D5" xr:uid="{504DE116-4C50-4705-9A3E-BE8293DC825F}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D5">
+    <sortCondition ref="A1:A5"/>
+  </sortState>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{229273D3-7C11-424D-8B36-626A8C193E57}" name="Device"/>
+    <tableColumn id="2" xr3:uid="{F532CE1E-E394-4538-AB6A-59CA790B7FB5}" name="Type"/>
+    <tableColumn id="3" xr3:uid="{44230D19-75FF-433E-BCF8-E7EB306CA978}" name="Description"/>
+    <tableColumn id="4" xr3:uid="{57D81849-A750-4DAF-8A0F-985F8B75A0B4}" name="Measure"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2460729E-6C27-47B1-8F39-2590CF2C50D6}" name="Table2" displayName="Table2" ref="A1:G27" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:G27" xr:uid="{2460729E-6C27-47B1-8F39-2590CF2C50D6}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G27">
+    <sortCondition ref="A1:A27"/>
+  </sortState>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{867C1170-48D8-40F4-B612-863059DA6E41}" name="Device"/>
+    <tableColumn id="2" xr3:uid="{5B68C7F2-DEA0-481D-B2E1-7F28F6AB10AB}" name="Port"/>
+    <tableColumn id="3" xr3:uid="{E80AE21E-0478-4333-B8BB-B0E0E760B476}" name="Direction"/>
+    <tableColumn id="4" xr3:uid="{CC7F72B7-A5AA-4B4D-9426-0BA0B52C402E}" name="X (um)"/>
+    <tableColumn id="5" xr3:uid="{EB39EA8D-2ED3-44A1-BBB1-74511C5F0CE3}" name="Y (um)"/>
+    <tableColumn id="6" xr3:uid="{90A213D5-77B1-4A82-900C-F18822FF7A9A}" name="Coupling"/>
+    <tableColumn id="7" xr3:uid="{67823E0A-DA1F-4F39-A856-FA26C19B2EBC}" name="Comments"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2F66197E-7C1E-41C7-B39D-EB7EFC540E5E}" name="Table4" displayName="Table4" ref="A1:E24" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:E24" xr:uid="{2F66197E-7C1E-41C7-B39D-EB7EFC540E5E}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E24">
+    <sortCondition ref="A1:A24"/>
+  </sortState>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{CFA7B5BF-1B63-4293-BCC7-DC0949EF0EB1}" name="Device"/>
+    <tableColumn id="2" xr3:uid="{206852AB-0D56-4FF3-8F24-08D2FAA89579}" name="Input"/>
+    <tableColumn id="3" xr3:uid="{6FF894C8-5677-44F3-8DA3-AF4FF6F8A57D}" name="Output"/>
+    <tableColumn id="4" xr3:uid="{A8D363A1-D727-4B55-A665-D6D5C71F3910}" name="Enabled"/>
+    <tableColumn id="5" xr3:uid="{B9343338-AB93-42A7-B737-3384971CA219}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -604,63 +727,66 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="45.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>63</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -670,70 +796,94 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="23.109375" customWidth="1"/>
+    <col min="4" max="4" width="12.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+      <c r="D3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>68</v>
+      </c>
+      <c r="D5" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D5" xr:uid="{C204D7B9-1C63-4579-AF0F-79A4D21FAC13}">
+      <formula1>"YES,NO"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -741,74 +891,79 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="10.5546875" customWidth="1"/>
+    <col min="7" max="7" width="12.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>31</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>635</v>
+        <v>952.5</v>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F2" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3">
+        <v>1016</v>
+      </c>
+      <c r="E3">
+        <v>300</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" t="s">
         <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3">
-        <v>698.5</v>
-      </c>
-      <c r="E3">
-        <v>100</v>
-      </c>
-      <c r="F3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G3" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -816,22 +971,22 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="D4">
-        <v>762</v>
+        <v>1079.5</v>
       </c>
       <c r="E4">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -839,22 +994,22 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D5">
-        <v>825.5</v>
+        <v>1143</v>
       </c>
       <c r="E5">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -862,573 +1017,941 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D6">
-        <v>889</v>
+        <v>1206.5</v>
       </c>
       <c r="E6">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F6" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="D7">
-        <v>952.5</v>
+        <v>1270</v>
       </c>
       <c r="E7">
         <v>300</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D8">
-        <v>1016</v>
+        <v>1333.5</v>
       </c>
       <c r="E8">
         <v>300</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D9">
-        <v>1079.5</v>
+        <v>1397</v>
       </c>
       <c r="E9">
         <v>300</v>
       </c>
       <c r="F9" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D10">
-        <v>1143</v>
+        <v>1460.5</v>
       </c>
       <c r="E10">
         <v>300</v>
       </c>
       <c r="F10" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D11">
-        <v>1206.5</v>
+        <v>1524</v>
       </c>
       <c r="E11">
         <v>300</v>
       </c>
       <c r="F11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" t="s">
         <v>34</v>
-      </c>
-      <c r="G11" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D12">
-        <v>1270</v>
+        <v>1587.5</v>
       </c>
       <c r="E12">
         <v>300</v>
       </c>
       <c r="F12" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D13">
-        <v>1333.5</v>
+        <v>1651</v>
       </c>
       <c r="E13">
         <v>300</v>
       </c>
       <c r="F13" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D14">
-        <v>1397</v>
+        <v>1714.5</v>
       </c>
       <c r="E14">
         <v>300</v>
       </c>
       <c r="F14" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D15">
-        <v>1460.5</v>
+        <v>1778</v>
       </c>
       <c r="E15">
         <v>300</v>
       </c>
       <c r="F15" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D16">
-        <v>1524</v>
+        <v>1841.5</v>
       </c>
       <c r="E16">
         <v>300</v>
       </c>
       <c r="F16" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G16" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D17">
-        <v>1587.5</v>
+        <v>1905</v>
       </c>
       <c r="E17">
         <v>300</v>
       </c>
       <c r="F17" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G17" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D18">
-        <v>1651</v>
+        <v>1968.5</v>
       </c>
       <c r="E18">
         <v>300</v>
       </c>
       <c r="F18" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="D19">
-        <v>1714.5</v>
+        <v>762</v>
       </c>
       <c r="E19">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F19" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="G19" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D20">
-        <v>1778</v>
+        <v>825.5</v>
       </c>
       <c r="E20">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F20" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="G20" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D21">
-        <v>1841.5</v>
+        <v>889</v>
       </c>
       <c r="E21">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F21" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="G21" t="s">
-        <v>66</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>8</v>
       </c>
       <c r="C22" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="D22">
-        <v>1905</v>
+        <v>2635</v>
       </c>
       <c r="E22">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F22" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="G22" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="B23" t="s">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="D23">
-        <v>1968.5</v>
+        <v>2698.5</v>
       </c>
       <c r="E23">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F23" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="G23" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="C24" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="D24">
-        <v>2635</v>
+        <v>2762</v>
       </c>
       <c r="E24">
         <v>100</v>
       </c>
       <c r="F24" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="G24" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="C25" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="D25">
-        <v>2698.5</v>
+        <v>2825.5</v>
       </c>
       <c r="E25">
         <v>100</v>
       </c>
       <c r="F25" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="G25" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="C26" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="D26">
-        <v>2762</v>
+        <v>635</v>
       </c>
       <c r="E26">
         <v>100</v>
       </c>
       <c r="F26" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D27">
-        <v>2825.5</v>
+        <v>698.5</v>
       </c>
       <c r="E27">
         <v>100</v>
       </c>
       <c r="F27" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="9.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
         <v>23</v>
       </c>
-      <c r="B4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5">
-        <v>4</v>
+      <c r="D5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" t="s">
+        <v>80</v>
+      </c>
+      <c r="E10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" t="s">
+        <v>80</v>
+      </c>
+      <c r="E13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" t="s">
+        <v>80</v>
+      </c>
+      <c r="E17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>80</v>
+      </c>
+      <c r="E18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>80</v>
+      </c>
+      <c r="E19" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" t="s">
+        <v>77</v>
+      </c>
+      <c r="E21" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" t="s">
+        <v>77</v>
+      </c>
+      <c r="E22" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" t="s">
+        <v>77</v>
+      </c>
+      <c r="E23" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>80</v>
+      </c>
+      <c r="E24" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D24" xr:uid="{9AB18791-B589-4AD7-92B7-A8C1A7808AF8}">
+      <formula1>"YES,NO"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>